<commit_message>
Delete gen_issue_tree_svg.py and add problem definition document for O2O strategy
</commit_message>
<xml_diff>
--- a/2026_Bain_Cup_Case_Data from Instant Retail Co.xlsx
+++ b/2026_Bain_Cup_Case_Data from Instant Retail Co.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://baincn-my.sharepoint.cn/personal/josh_zhu_bain_cn/Documents/Desktop/AC Recruiting/Bain Cup/26年贝恩杯/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zqnnnnnan/Library/Mobile Documents/com~apple~CloudDocs/Bainsight/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{5D99C1D3-6683-4779-8D03-F89B91560387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D77C7CB6-0007-4CBB-9DE0-4529886E2168}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A62B11A-A695-434E-B83B-23DF8E6F0491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12900" yWindow="760" windowWidth="16140" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="10城数据包" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="60">
   <si>
     <t>城市编号</t>
   </si>
@@ -204,17 +204,59 @@
   </si>
   <si>
     <t>2025年日均订单量（千单）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+      </rPr>
+      <t>常住人口</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>（万）</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>GDP</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>（亿）</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>人均可支配收入（元）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -222,6 +264,32 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="宋体"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -232,7 +300,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -255,18 +323,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -566,28 +651,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:W11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="4" width="28.5703125" customWidth="1"/>
-    <col min="5" max="5" width="27.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" customWidth="1"/>
-    <col min="7" max="7" width="30.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.5" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" customWidth="1"/>
+    <col min="4" max="4" width="28.5" customWidth="1"/>
+    <col min="5" max="5" width="27.6640625" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.6640625" customWidth="1"/>
     <col min="8" max="8" width="23" customWidth="1"/>
-    <col min="9" max="9" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="26" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="25" customWidth="1"/>
-    <col min="12" max="12" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="33.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="33.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="30" bestFit="1" customWidth="1"/>
-    <col min="17" max="19" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="19" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14" customWidth="1"/>
+    <col min="21" max="21" width="14.83203125" customWidth="1"/>
+    <col min="22" max="22" width="19.33203125" customWidth="1"/>
+    <col min="23" max="23" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:23" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -645,8 +734,18 @@
       <c r="S1" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="T1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="W1" s="2"/>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:23">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -704,8 +803,17 @@
       <c r="S2">
         <v>10</v>
       </c>
+      <c r="T2">
+        <v>903</v>
+      </c>
+      <c r="U2">
+        <v>9537.1200000000008</v>
+      </c>
+      <c r="V2">
+        <v>42230</v>
+      </c>
     </row>
-    <row r="3" spans="1:19">
+    <row r="3" spans="1:23">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -763,8 +871,17 @@
       <c r="S3">
         <v>12</v>
       </c>
+      <c r="T3">
+        <v>667.04</v>
+      </c>
+      <c r="U3">
+        <v>7800.37</v>
+      </c>
+      <c r="V3">
+        <v>57294</v>
+      </c>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:23">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -822,8 +939,17 @@
       <c r="S4">
         <v>10</v>
       </c>
+      <c r="T4">
+        <v>891.4</v>
+      </c>
+      <c r="U4">
+        <v>13094.87</v>
+      </c>
+      <c r="V4">
+        <v>52214</v>
+      </c>
     </row>
-    <row r="5" spans="1:19">
+    <row r="5" spans="1:23">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -881,8 +1007,17 @@
       <c r="S5">
         <v>12</v>
       </c>
+      <c r="T5">
+        <v>708.1</v>
+      </c>
+      <c r="U5">
+        <v>5819.8</v>
+      </c>
+      <c r="V5">
+        <v>35561</v>
+      </c>
     </row>
-    <row r="6" spans="1:19">
+    <row r="6" spans="1:23">
       <c r="A6" t="s">
         <v>32</v>
       </c>
@@ -940,8 +1075,17 @@
       <c r="S6">
         <v>12</v>
       </c>
+      <c r="T6">
+        <v>401</v>
+      </c>
+      <c r="U6">
+        <v>6120.27</v>
+      </c>
+      <c r="V6">
+        <v>36762</v>
+      </c>
     </row>
-    <row r="7" spans="1:19">
+    <row r="7" spans="1:23">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -999,8 +1143,17 @@
       <c r="S7">
         <v>12</v>
       </c>
+      <c r="T7">
+        <v>894</v>
+      </c>
+      <c r="U7">
+        <v>6000</v>
+      </c>
+      <c r="V7">
+        <v>37735</v>
+      </c>
     </row>
-    <row r="8" spans="1:19">
+    <row r="8" spans="1:23">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -1058,8 +1211,17 @@
       <c r="S8">
         <v>11</v>
       </c>
+      <c r="T8">
+        <v>611.67999999999995</v>
+      </c>
+      <c r="U8">
+        <v>6136.4</v>
+      </c>
+      <c r="V8">
+        <v>43849</v>
+      </c>
     </row>
-    <row r="9" spans="1:19">
+    <row r="9" spans="1:23">
       <c r="A9" t="s">
         <v>44</v>
       </c>
@@ -1117,8 +1279,17 @@
       <c r="S9">
         <v>12</v>
       </c>
+      <c r="T9">
+        <v>291.45999999999998</v>
+      </c>
+      <c r="U9">
+        <v>3728.62</v>
+      </c>
+      <c r="V9">
+        <v>51892</v>
+      </c>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:23">
       <c r="A10" t="s">
         <v>48</v>
       </c>
@@ -1176,8 +1347,17 @@
       <c r="S10">
         <v>12</v>
       </c>
+      <c r="T10">
+        <v>493.84</v>
+      </c>
+      <c r="U10">
+        <v>2517.39</v>
+      </c>
+      <c r="V10">
+        <v>34525</v>
+      </c>
     </row>
-    <row r="11" spans="1:19">
+    <row r="11" spans="1:23">
       <c r="A11" t="s">
         <v>51</v>
       </c>
@@ -1235,8 +1415,18 @@
       <c r="S11">
         <v>12</v>
       </c>
+      <c r="T11">
+        <v>897</v>
+      </c>
+      <c r="U11">
+        <v>4940.47</v>
+      </c>
+      <c r="V11">
+        <v>32128</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add initial configuration and workspace files for Obsidian setup
- Created app.json and appearance.json with default settings.
- Added core-plugins.json to enable essential plugins for enhanced functionality.
- Established workspace.json to define the layout and active tabs for user interface.
- Updated multiple Excel files with new data for analysis and reporting.
- Introduced slide-content.md for presentation on Instant Retail Co. strategy.
</commit_message>
<xml_diff>
--- a/2026_Bain_Cup_Case_Data from Instant Retail Co.xlsx
+++ b/2026_Bain_Cup_Case_Data from Instant Retail Co.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zqnnnnnan/Library/Mobile Documents/com~apple~CloudDocs/Bainsight/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A62B11A-A695-434E-B83B-23DF8E6F0491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12900" yWindow="760" windowWidth="16140" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="15120" windowHeight="14020"/>
   </bookViews>
   <sheets>
     <sheet name="10城数据包" sheetId="1" r:id="rId1"/>
@@ -33,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="61">
   <si>
     <t>城市编号</t>
   </si>
@@ -44,9 +38,18 @@
     <t>省份</t>
   </si>
   <si>
+    <t>Instant Retail Co.开城年份</t>
+  </si>
+  <si>
+    <t>2025年日均订单量（千单）</t>
+  </si>
+  <si>
     <t>订单年增速（%）</t>
   </si>
   <si>
+    <t>Instant Retail Co.市占率（%）</t>
+  </si>
+  <si>
     <t>平均客单价（元）</t>
   </si>
   <si>
@@ -81,129 +84,6 @@
   </si>
   <si>
     <t>订单结构_其他占比（%）</t>
-  </si>
-  <si>
-    <t>C1</t>
-  </si>
-  <si>
-    <t>徐州</t>
-  </si>
-  <si>
-    <t>江苏</t>
-  </si>
-  <si>
-    <t>年亏损约2,500万</t>
-  </si>
-  <si>
-    <t>C2</t>
-  </si>
-  <si>
-    <t>南昌</t>
-  </si>
-  <si>
-    <t>江西</t>
-  </si>
-  <si>
-    <t>年亏损约1,800万</t>
-  </si>
-  <si>
-    <t>C3</t>
-  </si>
-  <si>
-    <t>泉州</t>
-  </si>
-  <si>
-    <t>福建</t>
-  </si>
-  <si>
-    <t>基本盈亏平衡</t>
-  </si>
-  <si>
-    <t>C4</t>
-  </si>
-  <si>
-    <t>洛阳</t>
-  </si>
-  <si>
-    <t>河南</t>
-  </si>
-  <si>
-    <t>年亏损约2,200万</t>
-  </si>
-  <si>
-    <t>C5</t>
-  </si>
-  <si>
-    <t>宜昌</t>
-  </si>
-  <si>
-    <t>湖北</t>
-  </si>
-  <si>
-    <t>年亏损约1,200万</t>
-  </si>
-  <si>
-    <t>C6</t>
-  </si>
-  <si>
-    <t>南宁</t>
-  </si>
-  <si>
-    <t>广西</t>
-  </si>
-  <si>
-    <t>年亏损约2,000万</t>
-  </si>
-  <si>
-    <t>C7</t>
-  </si>
-  <si>
-    <t>惠州</t>
-  </si>
-  <si>
-    <t>广东</t>
-  </si>
-  <si>
-    <t>年亏损约1,000万</t>
-  </si>
-  <si>
-    <t>C8</t>
-  </si>
-  <si>
-    <t>威海</t>
-  </si>
-  <si>
-    <t>山东</t>
-  </si>
-  <si>
-    <t>小幅亏损，接近盈亏平衡</t>
-  </si>
-  <si>
-    <t>C9</t>
-  </si>
-  <si>
-    <t>桂林</t>
-  </si>
-  <si>
-    <t>年亏损约1,300万</t>
-  </si>
-  <si>
-    <t>C10</t>
-  </si>
-  <si>
-    <t>赣州</t>
-  </si>
-  <si>
-    <t>年亏损约1,500万</t>
-  </si>
-  <si>
-    <t>Instant Retail Co.开城年份</t>
-  </si>
-  <si>
-    <t>Instant Retail Co.市占率（%）</t>
-  </si>
-  <si>
-    <t>2025年日均订单量（千单）</t>
   </si>
   <si>
     <r>
@@ -211,7 +91,7 @@
         <b/>
         <sz val="11"/>
         <rFont val="宋体"/>
-        <family val="2"/>
+        <charset val="134"/>
       </rPr>
       <t>常住人口</t>
     </r>
@@ -220,15 +100,19 @@
         <b/>
         <sz val="11"/>
         <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
         <charset val="134"/>
       </rPr>
       <t>（万）</t>
     </r>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t>GDP</t>
     </r>
     <r>
@@ -236,39 +120,167 @@
         <b/>
         <sz val="11"/>
         <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
         <charset val="134"/>
       </rPr>
       <t>（亿）</t>
     </r>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>人均可支配收入（元）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>毛利率（</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>%</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）</t>
+    </r>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>徐州</t>
+  </si>
+  <si>
+    <t>江苏</t>
+  </si>
+  <si>
+    <t>年亏损约2,500万</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>南昌</t>
+  </si>
+  <si>
+    <t>江西</t>
+  </si>
+  <si>
+    <t>年亏损约1,800万</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>泉州</t>
+  </si>
+  <si>
+    <t>福建</t>
+  </si>
+  <si>
+    <t>基本盈亏平衡</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>洛阳</t>
+  </si>
+  <si>
+    <t>河南</t>
+  </si>
+  <si>
+    <t>年亏损约2,200万</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>宜昌</t>
+  </si>
+  <si>
+    <t>湖北</t>
+  </si>
+  <si>
+    <t>年亏损约1,200万</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t>南宁</t>
+  </si>
+  <si>
+    <t>广西</t>
+  </si>
+  <si>
+    <t>年亏损约2,000万</t>
+  </si>
+  <si>
+    <t>C7</t>
+  </si>
+  <si>
+    <t>惠州</t>
+  </si>
+  <si>
+    <t>广东</t>
+  </si>
+  <si>
+    <t>年亏损约1,000万</t>
+  </si>
+  <si>
+    <t>C8</t>
+  </si>
+  <si>
+    <t>威海</t>
+  </si>
+  <si>
+    <t>山东</t>
+  </si>
+  <si>
+    <t>小幅亏损，接近盈亏平衡</t>
+  </si>
+  <si>
+    <t>C9</t>
+  </si>
+  <si>
+    <t>桂林</t>
+  </si>
+  <si>
+    <t>年亏损约1,300万</t>
+  </si>
+  <si>
+    <t>C10</t>
+  </si>
+  <si>
+    <t>赣州</t>
+  </si>
+  <si>
+    <t>年亏损约1,500万</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="宋体"/>
-      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -276,31 +288,379 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="宋体"/>
-      <family val="2"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
+      <name val="宋体-简"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Microsoft YaHei"/>
-      <family val="2"/>
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -334,15 +694,260 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -350,17 +955,61 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -645,38 +1294,38 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:W11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.83653846153846" defaultRowHeight="16.8"/>
   <cols>
     <col min="2" max="2" width="13.5" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" customWidth="1"/>
+    <col min="3" max="3" width="10.6634615384615" customWidth="1"/>
     <col min="4" max="4" width="28.5" customWidth="1"/>
-    <col min="5" max="5" width="27.6640625" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.6640625" customWidth="1"/>
+    <col min="5" max="5" width="27.6634615384615" customWidth="1"/>
+    <col min="6" max="6" width="18.8365384615385" customWidth="1"/>
+    <col min="7" max="7" width="30.6634615384615" customWidth="1"/>
     <col min="8" max="8" width="23" customWidth="1"/>
-    <col min="9" max="9" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.6634615384615" customWidth="1"/>
+    <col min="10" max="10" width="26" customWidth="1"/>
     <col min="11" max="11" width="25" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="33.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="30" bestFit="1" customWidth="1"/>
-    <col min="17" max="19" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.8365384615385" customWidth="1"/>
+    <col min="13" max="13" width="22.3365384615385" customWidth="1"/>
+    <col min="14" max="14" width="16.1634615384615" customWidth="1"/>
+    <col min="15" max="15" width="33.3365384615385" customWidth="1"/>
+    <col min="16" max="16" width="30" customWidth="1"/>
+    <col min="17" max="19" width="25.5" customWidth="1"/>
     <col min="20" max="20" width="14" customWidth="1"/>
-    <col min="21" max="21" width="14.83203125" customWidth="1"/>
-    <col min="22" max="22" width="19.33203125" customWidth="1"/>
-    <col min="23" max="23" width="20.33203125" customWidth="1"/>
+    <col min="21" max="21" width="14.8365384615385" customWidth="1"/>
+    <col min="22" max="22" width="22.9038461538462" customWidth="1"/>
+    <col min="23" max="23" width="20.3365384615385" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="17">
+    <row r="1" ht="17" spans="1:23">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -687,73 +1336,75 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>54</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>56</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="W1" s="2"/>
+        <v>21</v>
+      </c>
+      <c r="W1" s="4" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="2" spans="1:23">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D2">
         <v>2019</v>
@@ -777,7 +1428,7 @@
         <v>4</v>
       </c>
       <c r="K2" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="L2">
         <v>95</v>
@@ -807,21 +1458,24 @@
         <v>903</v>
       </c>
       <c r="U2">
-        <v>9537.1200000000008</v>
+        <v>9537.12</v>
       </c>
       <c r="V2">
         <v>42230</v>
+      </c>
+      <c r="W2">
+        <v>0.75</v>
       </c>
     </row>
     <row r="3" spans="1:23">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="D3">
         <v>2020</v>
@@ -839,13 +1493,13 @@
         <v>55</v>
       </c>
       <c r="I3">
-        <v>9.8000000000000007</v>
+        <v>9.8</v>
       </c>
       <c r="J3">
         <v>4.5</v>
       </c>
       <c r="K3" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="L3">
         <v>80</v>
@@ -879,17 +1533,20 @@
       </c>
       <c r="V3">
         <v>57294</v>
+      </c>
+      <c r="W3">
+        <v>0.74</v>
       </c>
     </row>
     <row r="4" spans="1:23">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="D4">
         <v>2018</v>
@@ -907,13 +1564,13 @@
         <v>62</v>
       </c>
       <c r="I4">
-        <v>10.199999999999999</v>
+        <v>10.2</v>
       </c>
       <c r="J4">
         <v>3.5</v>
       </c>
       <c r="K4" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="L4">
         <v>110</v>
@@ -947,17 +1604,20 @@
       </c>
       <c r="V4">
         <v>52214</v>
+      </c>
+      <c r="W4">
+        <v>0.779</v>
       </c>
     </row>
     <row r="5" spans="1:23">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D5">
         <v>2020</v>
@@ -981,7 +1641,7 @@
         <v>4.8</v>
       </c>
       <c r="K5" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="L5">
         <v>70</v>
@@ -1015,17 +1675,20 @@
       </c>
       <c r="V5">
         <v>35561</v>
+      </c>
+      <c r="W5">
+        <v>0.688</v>
       </c>
     </row>
     <row r="6" spans="1:23">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D6">
         <v>2021</v>
@@ -1049,7 +1712,7 @@
         <v>4.2</v>
       </c>
       <c r="K6" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="L6">
         <v>55</v>
@@ -1083,17 +1746,20 @@
       </c>
       <c r="V6">
         <v>36762</v>
+      </c>
+      <c r="W6">
+        <v>0.737</v>
       </c>
     </row>
     <row r="7" spans="1:23">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D7">
         <v>2019</v>
@@ -1117,7 +1783,7 @@
         <v>4.3</v>
       </c>
       <c r="K7" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="L7">
         <v>85</v>
@@ -1151,17 +1817,20 @@
       </c>
       <c r="V7">
         <v>37735</v>
+      </c>
+      <c r="W7">
+        <v>0.73</v>
       </c>
     </row>
     <row r="8" spans="1:23">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D8">
         <v>2018</v>
@@ -1185,7 +1854,7 @@
         <v>3.8</v>
       </c>
       <c r="K8" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="L8">
         <v>100</v>
@@ -1212,24 +1881,27 @@
         <v>11</v>
       </c>
       <c r="T8">
-        <v>611.67999999999995</v>
+        <v>611.68</v>
       </c>
       <c r="U8">
         <v>6136.4</v>
       </c>
       <c r="V8">
         <v>43849</v>
+      </c>
+      <c r="W8">
+        <v>0.768</v>
       </c>
     </row>
     <row r="9" spans="1:23">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="D9">
         <v>2021</v>
@@ -1253,7 +1925,7 @@
         <v>3.5</v>
       </c>
       <c r="K9" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="L9">
         <v>45</v>
@@ -1280,24 +1952,27 @@
         <v>12</v>
       </c>
       <c r="T9">
-        <v>291.45999999999998</v>
+        <v>291.46</v>
       </c>
       <c r="U9">
         <v>3728.62</v>
       </c>
       <c r="V9">
         <v>51892</v>
+      </c>
+      <c r="W9">
+        <v>0.808</v>
       </c>
     </row>
     <row r="10" spans="1:23">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D10">
         <v>2022</v>
@@ -1318,10 +1993,10 @@
         <v>10.7</v>
       </c>
       <c r="J10">
-        <v>4.5999999999999996</v>
+        <v>4.6</v>
       </c>
       <c r="K10" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="L10">
         <v>40</v>
@@ -1355,17 +2030,20 @@
       </c>
       <c r="V10">
         <v>34525</v>
+      </c>
+      <c r="W10">
+        <v>0.681</v>
       </c>
     </row>
     <row r="11" spans="1:23">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="D11">
         <v>2022</v>
@@ -1386,10 +2064,10 @@
         <v>10.9</v>
       </c>
       <c r="J11">
-        <v>4.9000000000000004</v>
+        <v>4.9</v>
       </c>
       <c r="K11" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="L11">
         <v>38</v>
@@ -1424,15 +2102,12 @@
       <c r="V11">
         <v>32128</v>
       </c>
+      <c r="W11">
+        <v>0.649</v>
+      </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{47d9c042-e076-46f3-86c6-dfe85d7d78f5}" enabled="0" method="" siteId="{47d9c042-e076-46f3-86c6-dfe85d7d78f5}" removed="1"/>
-</clbl:labelList>
 </file>
</xml_diff>